<commit_message>
Enhance partner intake crosswalk documentation and update related scripts
- Updated `data/README.md` to include details about the new partner intake crosswalk and its seeding process.
- Expanded `docs/crosswalk-model.md` with a section on the partner crosswalk template, outlining its purpose and usage.
- Modified `docs/demographics-pilot-plan.md` to reflect the seeding of the partner crosswalk template.
- Updated `docs/excel-workbook-guide.md` to clarify the role of the Crosswalk_Template in mapping local codes to CHI standards.
- Adjusted `docs/operational-runbook.md` to include commands for seeding the partner crosswalk template.
- Enhanced `scripts/generate_intake_workbook.py` to integrate the partner crosswalk template into the workbook generation process.
- Regenerated binary files `chi-partner-intake-workbook.xlsx` and `chi-steward-workbook.xlsx` to reflect the latest changes.
</commit_message>
<xml_diff>
--- a/workbooks/chi-partner-intake-workbook.xlsx
+++ b/workbooks/chi-partner-intake-workbook.xlsx
@@ -14,10 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Inventory" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Values" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys_and_Relationships" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Questions" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHI_Curation_Bridge" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance_Load_Plan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crosswalk_Template" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys_and_Relationships" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open_Questions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHI_Curation_Bridge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance_Load_Plan" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -169,8 +170,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="chi_intake_table_index" displayName="chi_intake_table_index" ref="A1:D11" headerRowCount="1">
-  <autoFilter ref="A1:D11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="chi_intake_table_index" displayName="chi_intake_table_index" ref="A1:D12" headerRowCount="1">
+  <autoFilter ref="A1:D12"/>
   <tableColumns count="4">
     <tableColumn id="1" name="excel_table_name"/>
     <tableColumn id="2" name="sheet_tab"/>
@@ -181,9 +182,25 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="chi_intake_governance_load_plan" displayName="chi_intake_governance_load_plan" ref="A1:G2" headerRowCount="1">
+  <autoFilter ref="A1:G2"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="source_field_name"/>
+    <tableColumn id="2" name="approved_semantic_id"/>
+    <tableColumn id="3" name="target_governance_table"/>
+    <tableColumn id="4" name="target_column_or_purpose"/>
+    <tableColumn id="5" name="load_action"/>
+    <tableColumn id="6" name="dependencies_or_prereqs"/>
+    <tableColumn id="7" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="chi_intake_lookup_lists" displayName="chi_intake_lookup_lists" ref="A1:B7" headerRowCount="1">
-  <autoFilter ref="A1:B7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="chi_intake_lookup_lists" displayName="chi_intake_lookup_lists" ref="A1:B10" headerRowCount="1">
+  <autoFilter ref="A1:B10"/>
   <tableColumns count="2">
     <tableColumn id="1" name="field"/>
     <tableColumn id="2" name="allowed_values"/>
@@ -212,8 +229,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="chi_intake_field_inventory" displayName="chi_intake_field_inventory" ref="A1:L4" headerRowCount="1">
-  <autoFilter ref="A1:L4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="chi_intake_field_inventory" displayName="chi_intake_field_inventory" ref="A1:L5" headerRowCount="1">
+  <autoFilter ref="A1:L5"/>
   <tableColumns count="12">
     <tableColumn id="1" name="source_field_name"/>
     <tableColumn id="2" name="source_table_or_file"/>
@@ -248,7 +265,29 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="chi_intake_keys_relationships" displayName="chi_intake_keys_relationships" ref="A1:G2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="chi_intake_crosswalk_template" displayName="chi_intake_crosswalk_template" ref="A1:M8" headerRowCount="1">
+  <autoFilter ref="A1:M8"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="source_id"/>
+    <tableColumn id="2" name="source_field"/>
+    <tableColumn id="3" name="source_code"/>
+    <tableColumn id="4" name="source_display"/>
+    <tableColumn id="5" name="semantic_id"/>
+    <tableColumn id="6" name="target_code_system_oid"/>
+    <tableColumn id="7" name="target_code"/>
+    <tableColumn id="8" name="target_display"/>
+    <tableColumn id="9" name="mapping_type"/>
+    <tableColumn id="10" name="approval_status"/>
+    <tableColumn id="11" name="effective_from"/>
+    <tableColumn id="12" name="effective_to"/>
+    <tableColumn id="13" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="chi_intake_keys_relationships" displayName="chi_intake_keys_relationships" ref="A1:G2" headerRowCount="1">
   <autoFilter ref="A1:G2"/>
   <tableColumns count="7">
     <tableColumn id="1" name="record_type"/>
@@ -263,8 +302,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="chi_intake_open_questions" displayName="chi_intake_open_questions" ref="A1:E2" headerRowCount="1">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="chi_intake_open_questions" displayName="chi_intake_open_questions" ref="A1:E2" headerRowCount="1">
   <autoFilter ref="A1:E2"/>
   <tableColumns count="5">
     <tableColumn id="1" name="topic"/>
@@ -277,8 +316,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="chi_intake_curation_bridge" displayName="chi_intake_curation_bridge" ref="A1:L2" headerRowCount="1">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="chi_intake_curation_bridge" displayName="chi_intake_curation_bridge" ref="A1:L2" headerRowCount="1">
   <autoFilter ref="A1:L2"/>
   <tableColumns count="12">
     <tableColumn id="1" name="source_field_name"/>
@@ -293,22 +332,6 @@
     <tableColumn id="10" name="curation_disposition"/>
     <tableColumn id="11" name="needs_business_rule_review"/>
     <tableColumn id="12" name="chi_notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="chi_intake_governance_load_plan" displayName="chi_intake_governance_load_plan" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="source_field_name"/>
-    <tableColumn id="2" name="approved_semantic_id"/>
-    <tableColumn id="3" name="target_governance_table"/>
-    <tableColumn id="4" name="target_column_or_purpose"/>
-    <tableColumn id="5" name="load_action"/>
-    <tableColumn id="6" name="dependencies_or_prereqs"/>
-    <tableColumn id="7" name="notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -603,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -674,7 +697,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Document code lists in Code_Values and record joins in Keys_and_Relationships.</t>
+          <t>Document code lists in Code_Values; add crosswalk rows in Crosswalk_Template where you know local → standard mappings.</t>
         </is>
       </c>
     </row>
@@ -686,81 +709,93 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>Record joins in Keys_and_Relationships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  6.</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>Log blockers in Open_Questions, then review the Before you submit checklist on Intake_Guide.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Gather source-system information from a partner, then bridge into CHI governance.</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Table naming</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pattern: chi_intake_{artifact}. See Table_Index for sheet roles and who fills each table.</t>
+          <t>Gather source-system information from a partner, then bridge into CHI governance.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Intake_Guide</t>
+          <t>Table naming</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Partner entry sheet: intake flow steps, Field_Inventory column guide, and submission checklist.</t>
+          <t>Pattern: chi_intake_{artifact}. See Table_Index for sheet roles and who fills each table.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Who fills what</t>
+          <t>Intake_Guide</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Partner: Code_Values, Field_Inventory, Keys_and_Relationships, Open_Questions, Source_Summary. CHI: CHI_Curation_Bridge, Governance_Load_Plan.</t>
+          <t>Partner entry sheet: intake flow steps, Field_Inventory column guide, and submission checklist.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Allowed values</t>
+          <t>Who fills what</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Copy from Lookup_Lists instead of dropdowns (avoids Excel repair prompts).</t>
+          <t>Partner: Code_Values, Crosswalk_Template, Field_Inventory, Keys_and_Relationships, Open_Questions, Source_Summary. CHI: CHI_Curation_Bridge, Governance_Load_Plan.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Allowed values</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Copy from Lookup_Lists instead of dropdowns (avoids Excel repair prompts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Partners do not assign semantic_id, FHIR paths, USCDI mappings, or survivorship logic.</t>
         </is>
@@ -772,6 +807,80 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>question</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>resolution_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Identifiers</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Is PersonID stable across re-bookings and historical extracts?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Local Jail + CHI</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -894,7 +1003,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -988,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1110,12 +1219,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>chi_intake_keys_relationships</t>
+          <t>chi_intake_crosswalk_template</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Keys_and_Relationships</t>
+          <t>Crosswalk_Template</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1132,12 +1241,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>chi_intake_open_questions</t>
+          <t>chi_intake_keys_relationships</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Open_Questions</t>
+          <t>Keys_and_Relationships</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1154,34 +1263,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>chi_intake_curation_bridge</t>
+          <t>chi_intake_open_questions</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CHI_Curation_Bridge</t>
+          <t>Open_Questions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CHI bridge</t>
+          <t>Intake flow</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>chi_intake_governance_load_plan</t>
+          <t>chi_intake_curation_bridge</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Governance_Load_Plan</t>
+          <t>CHI_Curation_Bridge</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1198,42 +1307,64 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>chi_intake_lookup_lists</t>
+          <t>chi_intake_governance_load_plan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Lookup_Lists</t>
+          <t>Governance_Load_Plan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>CHI bridge</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>chi_intake_lookup_lists</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lookup_Lists</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>chi_intake_table_index</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Table_Index</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
@@ -1253,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1341,6 +1472,42 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>create_or_update</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mapping_type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>exact | rollup | exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>draft | Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>target_governance_table (crosswalk)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ddc-source_value_crosswalk (Source_Value_Crosswalk sheet in steward workbook)</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1464,12 +1631,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Keys_and_Relationships</t>
+          <t>Crosswalk_Template</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>How records join (booking to person, encounter to patient, etc.).</t>
+          <t>How your local codes map to CHI standards (example: GenderIdentity → Patient.gender_id). Replace example rows; keep source_id as partner_intake until CHI assigns yours.</t>
         </is>
       </c>
     </row>
@@ -1481,16 +1648,32 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>Keys_and_Relationships</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>How records join (booking to person, encounter to patient, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
           <t>Open_Questions</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Blockers and clarifications for CHI follow-up.</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -1686,19 +1869,26 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Keys_and_Relationships explains how person, encounter, and event records join.</t>
+          <t xml:space="preserve">  - Crosswalk_Template maps local codes to CHI semantic_id and standard target codes (see docs/partner-crosswalk-template.md).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Open_Questions has no unresolved blockers marked open without an owner.</t>
+          <t xml:space="preserve">  - Keys_and_Relationships explains how person, encounter, and event records join.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Open_Questions has no unresolved blockers marked open without an owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Example rows (jail booking sample) are replaced or clearly marked as examples.</t>
         </is>
@@ -1848,12 +2038,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -1861,7 +2051,7 @@
     <col width="38" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -2076,12 +2266,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2054-5</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>OMB race categories; see Code_Values if you maintain a local list</t>
+          <t>Local race list; map to CHI standards in Crosswalk_Template</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2102,6 +2292,68 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>Example demographics field. Add ethnicity, language, and sex fields the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>person.csv</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gender Identity</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Self-reported gender identity (not sex at birth / SexID)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FEMALE</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>See Crosswalk_Template — maps to Patient.gender_id, not birth sex</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>At intake when collected</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Distinct from SexID or administrative sex fields.</t>
         </is>
       </c>
     </row>
@@ -2208,6 +2460,518 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>source_field</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>source_code</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>source_display</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>semantic_id</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>target_code_system_oid</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>target_code</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>target_display</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>mapping_type</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>approval_status</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>effective_from</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>effective_to</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FEMALE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Female (self-reported)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.96</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>446141000124107</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Female gender identity</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Example: local export code → HL7 gender-identity minimum set. Not SexID / birth sex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MALE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Male (self-reported)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.96</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>446151000124109</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Male gender identity</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Distinct from administrative SexID on Patient.birth_sex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NONBINARY</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Non-binary</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.96</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>33791000087105</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Non-binary gender identity</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>CHI partner crosswalk template; replace source_id with assigned source_id after intake</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TWO_SPIRIT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Two-Spirit</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.96</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>33791000087105</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Non-binary gender identity</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>rollup</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Jurisdiction-specific label rolled to SNOMED minimum set; steward may refine after clinical review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DECLINE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Declined to answer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>http://terminology.hl7.org/CodeSystem/data-absent-reason</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>asked-declined</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Asked but declined</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Exclude from equity aggregates per survivorship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GenderIdentity</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Patient.gender_id</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.5.1008</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>UNK</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Treated as null at master level when source sends non-answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>partner_intake</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RaceCode</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Patient.race</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>urn:oid:2.16.840.1.113883.6.238</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2028-9</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Asian</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>rollup</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Pattern example only — replace with your local race code list; target must be governed CDCREC OMB rollup.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2300,78 +3064,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>topic</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>question</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>resolution_notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Identifiers</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Is PersonID stable across re-bookings and historical extracts?</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Local Jail + CHI</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>